<commit_message>
Discrepancy register: client wording for build impact, sources and questions; rebuilt workbook
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Registers/BIBS_Register_BRD-00_Discrepancies_and_Clarifications_v1.2.xlsx
+++ b/docs/deliverables/out/Programme/Registers/BIBS_Register_BRD-00_Discrepancies_and_Clarifications_v1.2.xlsx
@@ -1152,7 +1152,7 @@
     <row r="32">
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>Page numbers are PDF pages of the source files in docs/source-documents.</t>
+          <t>Page numbers are PDF pages of the source BRD files.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="C8" s="14" t="inlineStr">
         <is>
-          <t>Requirement ID, section and PDF page of the source file in docs/source-documents, for each BRD involved.</t>
+          <t>Requirement ID, section and PDF page of the source BRD, for each BRD involved.</t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr"/>
@@ -1368,12 +1368,12 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Impact (business / build / test)</t>
+          <t>Impact (business / system / test)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Effect on the business process, on what is built, and on testing.</t>
+          <t>Effect on the business process, on the system, and on testing.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr"/>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>What the project proposes, and builds as the default until BDOI answers.</t>
+          <t>What the project proposes, and applies as the default until BDOI answers.</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr"/>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Spec that raised the question (Cross-BRD: BDOI_CROSS_BRD_DECISIONS.md).</t>
+          <t>Requirements baseline that raised the question (Cross-BRD: the cross-BRD decisions).</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr"/>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>The item changes what is built or how data is structured, affects money (premium, commission, GL, remittance), regulatory compliance, security or access, or leaves a requirement without a testable result. Resolve before the FRS of the area is signed off.</t>
+          <t>The item changes what the system does or how data is structured, affects money (premium, commission, GL, remittance), regulatory compliance, security or access, or leaves a requirement without a testable result. Resolve before the FRS of the area is signed off.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>The item changes a rule, value, screen, report or test case, but a documented default can be built now and changed later by configuration or a small change.</t>
+          <t>The item changes a rule, value, screen, report or test case, but a documented default can apply now and be changed later by configuration or a small change.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>Document quality only (typing, numbering, headings, working notes, names). No effect on the build; correct it in the next BRD revision.</t>
+          <t>Document quality only (typing, numbering, headings, working notes, names). No effect on the system; correct it in the next BRD revision.</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>A value, list, layout or rule needed to build or test is missing or marked TBD.</t>
+          <t>A value, list, layout or rule needed to specify or test is missing or marked TBD.</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>The BRD differs from BIBS as built or designed, or assumes a legacy system (EBIX, QPS, ISYS) that BIBS replaces.</t>
+          <t>The BRD differs from BIBS as specified in the FRS, or assumes a legacy system (EBIX, QPS, ISYS) that BIBS replaces.</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="27" customHeight="1">
+    <row r="72" ht="15" customHeight="1">
       <c r="A72" s="21" t="inlineStr">
         <is>
           <t>BRD-0 CORE</t>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t>BDOI Core Replacement (umbrella): docs/source-documents/00 - BRD BDOI Core Replacement v01.pdf; baseline docs/requirements/BDOI_CORE_BRD_SPEC.md</t>
+          <t>BDOI Core Replacement (umbrella): 00 - BRD BDOI Core Replacement v01.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>New Business (NB): docs/source-documents/New Business (NB) BRD.pdf; baseline docs/requirements/BDOI_NB_BRD_SPEC.md</t>
+          <t>New Business (NB): New Business (NB) BRD.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="B74" s="12" t="inlineStr">
         <is>
-          <t>Operations: docs/source-documents/Operations.pdf; baseline docs/requirements/BDOI_OPS_BRD_SPEC.md</t>
+          <t>Operations: Operations.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>Product Maintenance: docs/source-documents/Product Maintenance.pdf; baseline docs/requirements/BDOI_PM_BRD_SPEC.md</t>
+          <t>Product Maintenance: Product Maintenance.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B76" s="12" t="inlineStr">
         <is>
-          <t>Collections (CLXN): docs/source-documents/Collections (CLXN) BRD.pdf; baseline docs/requirements/BDOI_CLXN_BRD_SPEC.md</t>
+          <t>Collections (CLXN): Collections (CLXN) BRD.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>Accounting, Disbursement and ACSL: docs/source-documents/Accounting, Disbursement, and Accounting Controls and Subsidiary Ledger BRD.zip; baseline docs/requirements/BDOI_ACCT_BRD_SPEC.md</t>
+          <t>Accounting, Disbursement and ACSL: Accounting, Disbursement, and Accounting Controls and Subsidiary Ledger BRD.zip; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="B78" s="12" t="inlineStr">
         <is>
-          <t>Renewal (RN): docs/source-documents/Renewal (RN) BRD.pdf; baseline docs/requirements/BDOI_RN_BRD_SPEC.md</t>
+          <t>Renewal (RN): Renewal (RN) BRD.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="B79" s="12" t="inlineStr">
         <is>
-          <t>Claims (CLM): docs/source-documents/Claims (CLM).PDF; baseline docs/requirements/BDOI_CLM_BRD_SPEC.md</t>
+          <t>Claims (CLM): Claims (CLM).PDF; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2374,11 +2374,11 @@
       </c>
       <c r="B80" s="12" t="inlineStr">
         <is>
-          <t>Employee Benefits (EB): docs/source-documents/Employee Benefits.pdf; baseline docs/requirements/BDOI_EB_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="27" customHeight="1">
+          <t>Employee Benefits (EB): Employee Benefits.pdf; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1">
       <c r="A81" s="21" t="inlineStr">
         <is>
           <t>BRD-9 CSF</t>
@@ -2386,11 +2386,11 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>Customer Servicing Facility (CSF): docs/source-documents/Customer Servicing Facility.PDF; baseline docs/requirements/BDOI_CSF_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="27" customHeight="1">
+          <t>Customer Servicing Facility (CSF): Customer Servicing Facility.PDF; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1">
       <c r="A82" s="21" t="inlineStr">
         <is>
           <t>BRD-10 SANC</t>
@@ -2398,11 +2398,11 @@
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t>Sanction Screening and Risk Profiling: docs/source-documents/Sanction Screening and Risk Profiling BRD.pdf; baseline docs/requirements/BDOI_SANC_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="27" customHeight="1">
+          <t>Sanction Screening and Risk Profiling: Sanction Screening and Risk Profiling BRD.pdf; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
       <c r="A83" s="21" t="inlineStr">
         <is>
           <t>BRD-11 UAM</t>
@@ -2410,11 +2410,11 @@
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t>User Access Maintenance (UAM): docs/source-documents/User Access Maintenance.pdf; baseline docs/requirements/BDOI_UAM_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="27" customHeight="1">
+          <t>User Access Maintenance (UAM): User Access Maintenance.pdf; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1">
       <c r="A84" s="21" t="inlineStr">
         <is>
           <t>BRD-12 SP</t>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="B84" s="12" t="inlineStr">
         <is>
-          <t>Submitted Policies (SP): docs/source-documents/BRD - Submitted Policies (with e-sig MCM 4.24.2026).pdf; baseline docs/requirements/BDOI_SP_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="27" customHeight="1">
+          <t>Submitted Policies (SP): BRD - Submitted Policies (with e-sig MCM 4.24.2026).pdf; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
       <c r="A85" s="21" t="inlineStr">
         <is>
           <t>BRD-13 DM</t>
@@ -2434,11 +2434,11 @@
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>Data Migration (draft v0.01): docs/source-documents/BRD - Data Migration - draft V0.01.pdf; baseline docs/requirements/BDOI_DM_BRD_SPEC.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="27" customHeight="1">
+          <t>Data Migration (draft v0.01): BRD - Data Migration - draft V0.01.pdf; with its requirements baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
       <c r="A86" s="21" t="inlineStr">
         <is>
           <t>Report List</t>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="B86" s="12" t="inlineStr">
         <is>
-          <t>Report List as of 27-Apr-2026: docs/source-documents/Report List as of APR-27-2026.pdf; baseline docs/requirements/BDOI_REPORT_LIST.md</t>
+          <t>Report List as of 27-Apr-2026: Report List as of APR-27-2026.pdf; with its requirements baseline</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>docs/requirements/BDOI_CROSS_BRD_DECISIONS.md (decisions D1-D8, questions XQ01-XQ13)</t>
+          <t>Cross-BRD decisions (decisions D1-D8, questions XQ01-XQ13)</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B88" s="12" t="inlineStr">
         <is>
-          <t>docs/architecture/PROGRAMME_ALIGNMENT.md (BDOI drop plan, timeline, IER workbook v20, integrations; questions IQ01-IQ35) and docs/architecture/DOCUMENT_STORAGE_DECISION.md (questions DSQ01-DSQ04)</t>
+          <t>Programme alignment (BDOI drop plan, timeline, IER workbook v20, integrations; questions IQ01-IQ35) and the document storage proposal (questions DSQ01-DSQ04)</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t>Each item was checked against the source page (text layer, or the rendered page for scanned pages) and cites it. Items come from the observations, NFR and open-question sections of the specs, the cross-BRD decisions, the Report List, and a comparison with BIBS as built or designed.</t>
+          <t>Each item was checked against the source page (text layer, or the rendered page for scanned pages) and cites it. Items come from the observations, NFR and open-question sections of the specs, the cross-BRD decisions, the Report List, and a comparison with BIBS as specified in the FRS.</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B92" s="12" t="inlineStr">
         <is>
-          <t>Edit docs/deliverables/src/registers/discrepancy_register.yaml and run python docs/deliverables/src/registers/build_discrepancy_register.py. Open questions are re-read from the specs at every build.</t>
+          <t>The register is re-issued with each update; open questions are refreshed from the requirements baselines at every issue.</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
     <row r="64">
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>The 15 items that most affect the build, money or compliance, in the order proposed for resolution.</t>
+          <t>The 15 items that most affect the system, money or compliance, in the order proposed for resolution.</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4012,7 @@
       <c r="G71" s="35" t="n"/>
       <c r="H71" s="14" t="inlineStr">
         <is>
-          <t>Build item ST0 / ST1 across every module that stores files.</t>
+          <t>Affects every module that stores files.</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="G4" s="37" t="inlineStr">
         <is>
-          <t>Impact (business / build / test)</t>
+          <t>Impact (business / system / test)</t>
         </is>
       </c>
       <c r="H4" s="37" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Business: walk-in and bank-referred prospects may not be quotable. Build: decides whether a prospect client code is created at quotation. Test: one of the two rows fails whichever rule is built.</t>
+          <t>Business: walk-in and bank-referred prospects may not be quotable. System: decides whether a prospect client code is created at quotation. Test: one of the two rows fails whichever rule applies.</t>
         </is>
       </c>
       <c r="H5" s="39" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>Build: the function is not traced to a governing requirement. Test: no acceptance criteria in the BRNB set.</t>
+          <t>System: the function is not traced to a governing requirement. Test: no acceptance criteria in the BRNB set.</t>
         </is>
       </c>
       <c r="H6" s="39" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Business: gross premium on quotations and invoices is wrong if the rate is wrong. Build: premium calculator and tax table. Test: expected premiums in test cases.</t>
+          <t>Business: gross premium on quotations and invoices is wrong if the rate is wrong. System: premium calculator and tax table. Test: expected premiums in test cases.</t>
         </is>
       </c>
       <c r="H9" s="39" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Business: Motor premium differs by 9 points of TSI. Build: motor rating rule. Test: expected premiums.</t>
+          <t>Business: Motor premium differs by 9 points of TSI. System: motor rating rule. Test: expected premiums.</t>
         </is>
       </c>
       <c r="H10" s="39" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Build: retention and archive rules. The baseline applies the addendum (later document).</t>
+          <t>System: retention and archive rules. The baseline applies the addendum (later document).</t>
         </is>
       </c>
       <c r="H11" s="39" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Build: session timer. Test: logout timing cases.</t>
+          <t>System: session timer. Test: logout timing cases.</t>
         </is>
       </c>
       <c r="H12" s="39" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Build: no owner for the report. Test: BRNB.018 cannot be accepted.</t>
+          <t>System: no owner for the report. Test: BRNB.018 cannot be accepted.</t>
         </is>
       </c>
       <c r="H13" s="39" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Build it in Renewal as a variant of the renewal listing (renewals booked after expiry).</t>
+          <t>Provide it in Renewal as a variant of the renewal listing (renewals booked after expiry).</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>Business: renewal production cannot be reported apart from new business. Build: shared change BT0 (account business type, invoice, report filters). Test: every booking and production report test.</t>
+          <t>Business: renewal production cannot be reported apart from new business. System: shared change BT0 (account business type, invoice, report filters). Test: every booking and production report test.</t>
         </is>
       </c>
       <c r="H14" s="39" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Build work item BT0 once for all three BRDs: business type on the account, carried to the invoice and used as a report filter.</t>
+          <t>One business type on the account (BT0) for all three BRDs, carried to the invoice and used as a report filter.</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Build: remittance extraction screen. The addendum governs.</t>
+          <t>System: remittance extraction screen. The addendum governs.</t>
         </is>
       </c>
       <c r="H15" s="39" t="inlineStr">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Build exclusion only (no edit of financial fields), per Addendum 1.</t>
+          <t>Exclusion only (no edit of financial fields), per Addendum 1.</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Build: one function, two IDs. Test: two rows cite one screen.</t>
+          <t>System: one function, two IDs. Test: two rows cite one screen.</t>
         </is>
       </c>
       <c r="H16" s="39" t="inlineStr">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>Build the Endorsement Slip once, available to Marketing and Adjustment users.</t>
+          <t>One Endorsement Slip, available to Marketing and Adjustment users.</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Business: incentive income may be computed twice or on the wrong lines. Build: one computation owner. Test: incentive amounts.</t>
+          <t>Business: incentive income may be computed twice or on the wrong lines. System: one computation owner. Test: incentive amounts.</t>
         </is>
       </c>
       <c r="H17" s="39" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Business: small balances post to different GL accounts. Build: cashiering and adjustment rules. Test: boundary cases at 10.00.</t>
+          <t>Business: small balances post to different GL accounts. System: cashiering and adjustment rules. Test: boundary cases at 10.00.</t>
         </is>
       </c>
       <c r="H18" s="39" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>Business: remittance to insurers is capped or withheld. Build: remittance validation. Test: expected result differs.</t>
+          <t>Business: remittance to insurers is capped or withheld. System: remittance validation. Test: expected result differs.</t>
         </is>
       </c>
       <c r="H19" s="39" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>Build: remittance status model. Test: status transitions.</t>
+          <t>System: remittance status model. Test: status transitions.</t>
         </is>
       </c>
       <c r="H20" s="39" t="inlineStr">
@@ -5760,7 +5760,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Business: number of ORs issued for commission. Build: OR generation. Test: OR count.</t>
+          <t>Business: number of ORs issued for commission. System: OR generation. Test: OR count.</t>
         </is>
       </c>
       <c r="H21" s="39" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>Business: approval and premium may be skipped. Build: endorsement type list. Test: endorsement cases.</t>
+          <t>Business: approval and premium may be skipped. System: endorsement type list. Test: endorsement cases.</t>
         </is>
       </c>
       <c r="H22" s="39" t="inlineStr">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>Build: defaults must be assumed. Test: no expected values.</t>
+          <t>System: defaults must be assumed. Test: no expected values.</t>
         </is>
       </c>
       <c r="H23" s="39" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>Build each as a parameter or list with a documented default.</t>
+          <t>Each as a parameter or list with a documented default.</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>Build: upload screen vs batch intake. Test: file intake cases.</t>
+          <t>System: upload screen vs batch intake. Test: file intake cases.</t>
         </is>
       </c>
       <c r="H24" s="39" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>Build: in-app interfaces instead of external integrations.</t>
+          <t>System: in-app interfaces instead of external integrations.</t>
         </is>
       </c>
       <c r="H26" s="39" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Build: the Marketing screens stay in the Operations build.</t>
+          <t>System: the Marketing screens stay in Operations.</t>
         </is>
       </c>
       <c r="H27" s="39" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>Build: sizing assumed from BRD-1. Test: no volume targets for performance tests.</t>
+          <t>System: sizing assumed from BRD-1. Test: no volume targets for performance tests.</t>
         </is>
       </c>
       <c r="H29" s="39" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>Business: two owners for one process. Build: risk of two payment intakes and two endorsement paths. Test: duplicated cases.</t>
+          <t>Business: two owners for one process. System: risk of two payment intakes and two endorsement paths. Test: duplicated cases.</t>
         </is>
       </c>
       <c r="H31" s="39" t="inlineStr">
@@ -6599,7 +6599,7 @@
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>Business: GL entries for CWT unclear. Build: posting rules. Test: GL expected entries.</t>
+          <t>Business: GL entries for CWT unclear. System: posting rules. Test: GL expected entries.</t>
         </is>
       </c>
       <c r="H32" s="39" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>Business: a renewal could be repriced after the RA without client evidence. Build: renewal acceptance evidence.</t>
+          <t>Business: a renewal could be repriced after the RA without client evidence. System: renewal acceptance evidence.</t>
         </is>
       </c>
       <c r="H34" s="39" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="J35" s="12" t="inlineStr">
         <is>
-          <t>None for the build.</t>
+          <t>None for the system.</t>
         </is>
       </c>
       <c r="K35" s="12" t="inlineStr">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="G38" s="12" t="inlineStr">
         <is>
-          <t>Build: two reports with one name. Test: wrong report tested.</t>
+          <t>System: two reports with one name. Test: wrong report tested.</t>
         </is>
       </c>
       <c r="H38" s="39" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>Build: role-to-action matrix (PMADD05) has no agreed content. Test: access tests.</t>
+          <t>System: role-to-action matrix (PMADD05) has no agreed content. Test: access tests.</t>
         </is>
       </c>
       <c r="H39" s="39" t="inlineStr">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>Build: scope of product maintenance for non-package products is undefined.</t>
+          <t>System: scope of product maintenance for non-package products is undefined.</t>
         </is>
       </c>
       <c r="H40" s="39" t="inlineStr">
@@ -7284,7 +7284,7 @@
       </c>
       <c r="G41" s="12" t="inlineStr">
         <is>
-          <t>Business: incentive income and pass-on to branches. Build: one incentive model across modules. Test: no expected values.</t>
+          <t>Business: incentive income and pass-on to branches. System: one incentive model across modules. Test: no expected values.</t>
         </is>
       </c>
       <c r="H41" s="39" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="G43" s="12" t="inlineStr">
         <is>
-          <t>Business: scope of four requirements unclear. Build: rows designed as Draft. Test: no approved criteria.</t>
+          <t>Business: scope of four requirements unclear. System: rows specified as Draft. Test: no approved criteria.</t>
         </is>
       </c>
       <c r="H43" s="39" t="inlineStr">
@@ -7453,7 +7453,7 @@
       </c>
       <c r="J43" s="12" t="inlineStr">
         <is>
-          <t>Build BRCLXN.061-064 only after BDOI confirms them.</t>
+          <t>Deliver BRCLXN.061-064 only after BDOI confirms them.</t>
         </is>
       </c>
       <c r="K43" s="12" t="inlineStr">
@@ -7588,7 +7588,7 @@
       </c>
       <c r="G45" s="12" t="inlineStr">
         <is>
-          <t>Build: grain of the collection list and the threshold rule (BRCLXN.003). Test: list totals.</t>
+          <t>System: grain of the collection list and the threshold rule (BRCLXN.003). Test: list totals.</t>
         </is>
       </c>
       <c r="H45" s="39" t="inlineStr">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>Traceability only; the BOOKER field is built.</t>
+          <t>Traceability only; the BOOKER field is in BIBS.</t>
         </is>
       </c>
       <c r="H46" s="39" t="inlineStr">
@@ -7742,7 +7742,7 @@
       </c>
       <c r="G47" s="12" t="inlineStr">
         <is>
-          <t>Build: exports allowed or not. Test: export cases.</t>
+          <t>System: exports allowed or not. Test: export cases.</t>
         </is>
       </c>
       <c r="H47" s="39" t="inlineStr">
@@ -7819,7 +7819,7 @@
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>Security: session policy. Build: session registry. Test: multi-device login cases.</t>
+          <t>Security: session policy. System: session registry. Test: multi-device login cases.</t>
         </is>
       </c>
       <c r="H48" s="39" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="J48" s="12" t="inlineStr">
         <is>
-          <t>Session log built; the single-device rule is enforced only after BDOI confirms it (parameter, off by default).</t>
+          <t>Session log kept; the single-device rule is enforced only after BDOI confirms it (parameter, off by default).</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="G49" s="12" t="inlineStr">
         <is>
-          <t>Security: segregation of duties. Build: role assignment rule.</t>
+          <t>Security: segregation of duties. System: role assignment rule.</t>
         </is>
       </c>
       <c r="H49" s="39" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>Build: validation of invoice numbers during migration. Test: field mapping.</t>
+          <t>System: validation of invoice numbers during migration. Test: field mapping.</t>
         </is>
       </c>
       <c r="H50" s="39" t="inlineStr">
@@ -8142,7 +8142,7 @@
       </c>
       <c r="J52" s="12" t="inlineStr">
         <is>
-          <t>None for the build.</t>
+          <t>None for the system.</t>
         </is>
       </c>
       <c r="K52" s="12" t="inlineStr">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="G56" s="12" t="inlineStr">
         <is>
-          <t>Build: mandatory fields of the RRF / RFP. Test: field validations.</t>
+          <t>System: mandatory fields of the RRF / RFP. Test: field validations.</t>
         </is>
       </c>
       <c r="H56" s="39" t="inlineStr">
@@ -8573,7 +8573,7 @@
       </c>
       <c r="G58" s="12" t="inlineStr">
         <is>
-          <t>Business: month-end close. Build: closing validation. Test: closing-date cases.</t>
+          <t>Business: month-end close. System: closing validation. Test: closing-date cases.</t>
         </is>
       </c>
       <c r="H58" s="39" t="inlineStr">
@@ -8650,7 +8650,7 @@
       </c>
       <c r="G59" s="12" t="inlineStr">
         <is>
-          <t>Build: reports with no data source in BIBS. Test: report scope.</t>
+          <t>System: reports with no data source in BIBS. Test: report scope.</t>
         </is>
       </c>
       <c r="H59" s="39" t="inlineStr">
@@ -8727,7 +8727,7 @@
       </c>
       <c r="G60" s="12" t="inlineStr">
         <is>
-          <t>Build: bank account master and funding flow. Test: funding cases.</t>
+          <t>System: bank account master and funding flow. Test: funding cases.</t>
         </is>
       </c>
       <c r="H60" s="39" t="inlineStr">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="G61" s="12" t="inlineStr">
         <is>
-          <t>Build: HA design. Test: availability cannot be verified at 100%.</t>
+          <t>System: HA design. Test: availability cannot be verified at 100%.</t>
         </is>
       </c>
       <c r="H61" s="39" t="inlineStr">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="G62" s="12" t="inlineStr">
         <is>
-          <t>Business: BIR invoice uniqueness vs one reference per policy. Build: invoice numbering and sub-ledger. Test: ACSL reconciliation.</t>
+          <t>Business: BIR invoice uniqueness vs one reference per policy. System: invoice numbering and sub-ledger. Test: ACSL reconciliation.</t>
         </is>
       </c>
       <c r="H62" s="39" t="inlineStr">
@@ -8958,7 +8958,7 @@
       </c>
       <c r="G63" s="12" t="inlineStr">
         <is>
-          <t>Build: role grants. Test: access tests.</t>
+          <t>System: role grants. Test: access tests.</t>
         </is>
       </c>
       <c r="H63" s="39" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="J63" s="12" t="inlineStr">
         <is>
-          <t>Roles built from the scans; BDOI confirms.</t>
+          <t>Roles taken from the scans; BDOI confirms.</t>
         </is>
       </c>
       <c r="K63" s="12" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
-          <t>None on the build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H64" s="39" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="G65" s="12" t="inlineStr">
         <is>
-          <t>None on the build; shows the text was edited after the May 2025 signature.</t>
+          <t>None on the system; shows the text was edited after the May 2025 signature.</t>
         </is>
       </c>
       <c r="H65" s="39" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="G66" s="12" t="inlineStr">
         <is>
-          <t>Business: where AOs record dispositions. Build: disposition screens and upload. Test: both paths.</t>
+          <t>Business: where AOs record dispositions. System: disposition screens and upload. Test: both paths.</t>
         </is>
       </c>
       <c r="H66" s="39" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="J66" s="12" t="inlineStr">
         <is>
-          <t>Build both: online disposition for AOs and batch upload for bulk segments (CLG, insurer files).</t>
+          <t>Provide both: online disposition for AOs and batch upload for bulk segments (CLG, insurer files).</t>
         </is>
       </c>
       <c r="K66" s="12" t="inlineStr">
@@ -9258,7 +9258,7 @@
       </c>
       <c r="G67" s="12" t="inlineStr">
         <is>
-          <t>Business: control over renewal start. Build: workflow triggers. Test: STP scenarios.</t>
+          <t>Business: control over renewal start. System: workflow triggers. Test: STP scenarios.</t>
         </is>
       </c>
       <c r="H67" s="39" t="inlineStr">
@@ -9335,7 +9335,7 @@
       </c>
       <c r="G68" s="12" t="inlineStr">
         <is>
-          <t>Build: reminder schedule. Test: reminder dates.</t>
+          <t>System: reminder schedule. Test: reminder dates.</t>
         </is>
       </c>
       <c r="H68" s="39" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>Build: role of the Processing Officer; RA protection. Test: access and encryption cases.</t>
+          <t>System: role of the Processing Officer; RA protection. Test: access and encryption cases.</t>
         </is>
       </c>
       <c r="H70" s="39" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="G71" s="12" t="inlineStr">
         <is>
-          <t>Build: edit lock. Test: expected result inverted.</t>
+          <t>System: edit lock. Test: expected result inverted.</t>
         </is>
       </c>
       <c r="H71" s="39" t="inlineStr">
@@ -9723,7 +9723,7 @@
       </c>
       <c r="J73" s="12" t="inlineStr">
         <is>
-          <t>None for the build.</t>
+          <t>None for the system.</t>
         </is>
       </c>
       <c r="K73" s="12" t="inlineStr">
@@ -9781,7 +9781,7 @@
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>Build: counters cannot be computed. Test: counter values.</t>
+          <t>System: counters cannot be computed. Test: counter values.</t>
         </is>
       </c>
       <c r="H74" s="39" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="G75" s="12" t="inlineStr">
         <is>
-          <t>Build: no NFR values for Renewal. Test: no targets.</t>
+          <t>System: no NFR values for Renewal. Test: no targets.</t>
         </is>
       </c>
       <c r="H75" s="39" t="inlineStr">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="G76" s="12" t="inlineStr">
         <is>
-          <t>Build: recipient policy for RA e-mails. Test: sending rules.</t>
+          <t>System: recipient policy for RA e-mails. Test: sending rules.</t>
         </is>
       </c>
       <c r="H76" s="39" t="inlineStr">
@@ -10012,7 +10012,7 @@
       </c>
       <c r="G77" s="12" t="inlineStr">
         <is>
-          <t>Build: reason list vs tag. Test: NFR letter trigger.</t>
+          <t>System: reason list vs tag. Test: NFR letter trigger.</t>
         </is>
       </c>
       <c r="H77" s="39" t="inlineStr">
@@ -10089,7 +10089,7 @@
       </c>
       <c r="G78" s="12" t="inlineStr">
         <is>
-          <t>Build: grid pattern. Test: large list performance.</t>
+          <t>System: grid pattern. Test: large list performance.</t>
         </is>
       </c>
       <c r="H78" s="39" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="G79" s="12" t="inlineStr">
         <is>
-          <t>Business: first-year renewals of legacy policies could be missed. Build: one-time load of expiring policies. Test: renewal list completeness.</t>
+          <t>Business: first-year renewals of legacy policies could be missed. System: one-time load of expiring policies. Test: renewal list completeness.</t>
         </is>
       </c>
       <c r="H79" s="39" t="inlineStr">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="G80" s="12" t="inlineStr">
         <is>
-          <t>None on the build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H80" s="39" t="inlineStr">
@@ -10389,7 +10389,7 @@
       </c>
       <c r="G82" s="12" t="inlineStr">
         <is>
-          <t>Business: claim closure and reporting. Build: status and settlement model. Test: closure cases.</t>
+          <t>Business: claim closure and reporting. System: status and settlement model. Test: closure cases.</t>
         </is>
       </c>
       <c r="H82" s="39" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="G83" s="12" t="inlineStr">
         <is>
-          <t>Build: closure permissions. Test: access cases.</t>
+          <t>System: closure permissions. Test: access cases.</t>
         </is>
       </c>
       <c r="H83" s="39" t="inlineStr">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Build: retention rules; whether the values are binding. Test: purge cases.</t>
+          <t>System: retention rules; whether the values are binding. Test: purge cases.</t>
         </is>
       </c>
       <c r="H84" s="39" t="inlineStr">
@@ -10615,12 +10615,12 @@
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>The BRD asks for "a facility in eBIX" and assumes "the existing claims module is functional and can be enhanced"; assumption 3: "Data migration and integration with existing systems will be seamless". In BIBS the broker claims module is a new build; the platform's insurer-side claims module does not fit a broker.</t>
+          <t>The BRD asks for "a facility in eBIX" and assumes "the existing claims module is functional and can be enhanced"; assumption 3: "Data migration and integration with existing systems will be seamless". In BIBS the broker claims module is a new module; the platform's insurer-side claims module does not fit a broker.</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr">
         <is>
-          <t>Build: new module; claims history must be migrated. Test: migration.</t>
+          <t>System: new module; claims history must be migrated. Test: migration.</t>
         </is>
       </c>
       <c r="H85" s="39" t="inlineStr">
@@ -10697,7 +10697,7 @@
       </c>
       <c r="G86" s="12" t="inlineStr">
         <is>
-          <t>None on the build; acronyms need a glossary.</t>
+          <t>None on the system; acronyms need a glossary.</t>
         </is>
       </c>
       <c r="H86" s="39" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="G87" s="12" t="inlineStr">
         <is>
-          <t>Business: scope baseline. Build: BRCLM.037-043 are baselined in scope.</t>
+          <t>Business: scope baseline. System: BRCLM.037-043 are baselined in scope.</t>
         </is>
       </c>
       <c r="H87" s="39" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="G88" s="12" t="inlineStr">
         <is>
-          <t>Build: report layouts and delivery. Test: report columns.</t>
+          <t>System: report layouts and delivery. Test: report columns.</t>
         </is>
       </c>
       <c r="H88" s="39" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="G89" s="12" t="inlineStr">
         <is>
-          <t>Business: valid claims could be blocked. Build: premium validation rule. Test: claim intake cases.</t>
+          <t>Business: valid claims could be blocked. System: premium validation rule. Test: claim intake cases.</t>
         </is>
       </c>
       <c r="H89" s="39" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Business: cash handling. Build: Cashiering and Disbursement flows only if money passes through BDOI. Test: settlement cases.</t>
+          <t>Business: cash handling. System: Cashiering and Disbursement flows only if money passes through BDOI. Test: settlement cases.</t>
         </is>
       </c>
       <c r="H90" s="39" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="G91" s="12" t="inlineStr">
         <is>
-          <t>Build: RA schedule. Test: RA dates.</t>
+          <t>System: RA schedule. Test: RA dates.</t>
         </is>
       </c>
       <c r="H91" s="39" t="inlineStr">
@@ -11159,7 +11159,7 @@
       </c>
       <c r="G92" s="12" t="inlineStr">
         <is>
-          <t>Build: BOR validation. Test: renewal with BOR.</t>
+          <t>System: BOR validation. Test: renewal with BOR.</t>
         </is>
       </c>
       <c r="H92" s="39" t="inlineStr">
@@ -11236,7 +11236,7 @@
       </c>
       <c r="G93" s="12" t="inlineStr">
         <is>
-          <t>Build: none (OUT).</t>
+          <t>System: none (OUT).</t>
         </is>
       </c>
       <c r="H93" s="39" t="inlineStr">
@@ -11317,7 +11317,7 @@
       </c>
       <c r="G94" s="12" t="inlineStr">
         <is>
-          <t>Build: approval steps. Test: no criteria.</t>
+          <t>System: approval steps. Test: no criteria.</t>
         </is>
       </c>
       <c r="H94" s="39" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="G96" s="12" t="inlineStr">
         <is>
-          <t>Build: portal sizing. Test: no response-time target.</t>
+          <t>System: portal sizing. Test: no response-time target.</t>
         </is>
       </c>
       <c r="H96" s="39" t="inlineStr">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="G97" s="12" t="inlineStr">
         <is>
-          <t>Business: booking of member movements. Build: adjustment booking rule.</t>
+          <t>Business: booking of member movements. System: adjustment booking rule.</t>
         </is>
       </c>
       <c r="H97" s="39" t="inlineStr">
@@ -11621,7 +11621,7 @@
       </c>
       <c r="G98" s="12" t="inlineStr">
         <is>
-          <t>Business: Data Privacy Act exposure. Build: access classes and masking. Test: privacy tests.</t>
+          <t>Business: Data Privacy Act exposure. System: access classes and masking. Test: privacy tests.</t>
         </is>
       </c>
       <c r="H98" s="39" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="G99" s="12" t="inlineStr">
         <is>
-          <t>None on the build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H99" s="39" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="G100" s="12" t="inlineStr">
         <is>
-          <t>Security: internet-facing access. Build: portal realm and user provisioning. Test: security tests.</t>
+          <t>Security: internet-facing access. System: portal realm and user provisioning. Test: security tests.</t>
         </is>
       </c>
       <c r="H100" s="39" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="G101" s="12" t="inlineStr">
         <is>
-          <t>Build: catalog party type and commission rates for HMO providers.</t>
+          <t>System: catalog party type and commission rates for HMO providers.</t>
         </is>
       </c>
       <c r="H101" s="39" t="inlineStr">
@@ -12148,7 +12148,7 @@
       </c>
       <c r="G105" s="12" t="inlineStr">
         <is>
-          <t>Build: status mapping. Test: expected status.</t>
+          <t>System: status mapping. Test: expected status.</t>
         </is>
       </c>
       <c r="H105" s="39" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>Build: backup and WAL archiving design for the whole platform. Test: recovery tests.</t>
+          <t>System: backup and WAL archiving design for the whole platform. Test: recovery tests.</t>
         </is>
       </c>
       <c r="H106" s="39" t="inlineStr">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="G107" s="12" t="inlineStr">
         <is>
-          <t>Build: maintenance scheduling.</t>
+          <t>System: maintenance scheduling.</t>
         </is>
       </c>
       <c r="H107" s="39" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="G108" s="12" t="inlineStr">
         <is>
-          <t>Build: write-back interface to legacy systems. Test: coexistence cases.</t>
+          <t>System: write-back interface to legacy systems. Test: coexistence cases.</t>
         </is>
       </c>
       <c r="H108" s="39" t="inlineStr">
@@ -12606,7 +12606,7 @@
       </c>
       <c r="G111" s="12" t="inlineStr">
         <is>
-          <t>Build: re-assignment permission. Test: access cases.</t>
+          <t>System: re-assignment permission. Test: access cases.</t>
         </is>
       </c>
       <c r="H111" s="39" t="inlineStr">
@@ -12683,7 +12683,7 @@
       </c>
       <c r="G112" s="12" t="inlineStr">
         <is>
-          <t>Build: committee approval step. Test: approval cases.</t>
+          <t>System: committee approval step. Test: approval cases.</t>
         </is>
       </c>
       <c r="H112" s="39" t="inlineStr">
@@ -12760,7 +12760,7 @@
       </c>
       <c r="G113" s="12" t="inlineStr">
         <is>
-          <t>Compliance: PEP coverage for individuals. Build: list sources.</t>
+          <t>Compliance: PEP coverage for individuals. System: list sources.</t>
         </is>
       </c>
       <c r="H113" s="39" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="G114" s="12" t="inlineStr">
         <is>
-          <t>Build: sizing and role provisioning. Test: load tests.</t>
+          <t>System: sizing and role provisioning. Test: load tests.</t>
         </is>
       </c>
       <c r="H114" s="39" t="inlineStr">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="G115" s="12" t="inlineStr">
         <is>
-          <t>Compliance scope. Build: list types and review templates.</t>
+          <t>Compliance scope. System: list types and review templates.</t>
         </is>
       </c>
       <c r="H115" s="39" t="inlineStr">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="G116" s="12" t="inlineStr">
         <is>
-          <t>Compliance: business with a possible sanctioned party. Build: client compliance gate. Test: blocking cases.</t>
+          <t>Compliance: business with a possible sanctioned party. System: client compliance gate. Test: blocking cases.</t>
         </is>
       </c>
       <c r="H116" s="39" t="inlineStr">
@@ -13006,7 +13006,7 @@
       </c>
       <c r="J116" s="12" t="inlineStr">
         <is>
-          <t>Warn by banner; a block is built behind a parameter, off by default.</t>
+          <t>Warn by banner; a block is available behind a parameter, off by default.</t>
         </is>
       </c>
       <c r="K116" s="12" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="G118" s="12" t="inlineStr">
         <is>
-          <t>Build: whether one access process covers every BIBS module and persona.</t>
+          <t>System: whether one access process covers every BIBS module and persona.</t>
         </is>
       </c>
       <c r="H118" s="39" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="G119" s="12" t="inlineStr">
         <is>
-          <t>Test: acceptance criteria must be written by the project. Build: NFR values unknown.</t>
+          <t>Test: acceptance criteria must be written by the project. System: NFR values unknown.</t>
         </is>
       </c>
       <c r="H119" s="39" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="G121" s="12" t="inlineStr">
         <is>
-          <t>Build: FOR_IMPLEMENTATION step for group profiles. Test: approval cases.</t>
+          <t>System: FOR_IMPLEMENTATION step for group profiles. Test: approval cases.</t>
         </is>
       </c>
       <c r="H121" s="39" t="inlineStr">
@@ -13449,7 +13449,7 @@
       </c>
       <c r="G122" s="12" t="inlineStr">
         <is>
-          <t>Build: user ID validation. Test: user creation.</t>
+          <t>System: user ID validation. Test: user creation.</t>
         </is>
       </c>
       <c r="H122" s="39" t="inlineStr">
@@ -13521,12 +13521,12 @@
       </c>
       <c r="F123" s="12" t="inlineStr">
         <is>
-          <t>NFR 6 requires logging of user log-in and log-out. BIBS records log-in and failed log-in, but has no log-out endpoint, so log-out is not recorded.</t>
+          <t>NFR 6 requires logging of user log-in and log-out. The session log must record the log-out as well as the log-in and failed log-in.</t>
         </is>
       </c>
       <c r="G123" s="12" t="inlineStr">
         <is>
-          <t>Audit: session history incomplete. Build: log-out endpoint and session log.</t>
+          <t>Audit: session history complete only when the log-out is recorded. System: log-out recorded in the session log.</t>
         </is>
       </c>
       <c r="H123" s="39" t="inlineStr">
@@ -13680,7 +13680,7 @@
       </c>
       <c r="G125" s="12" t="inlineStr">
         <is>
-          <t>Build: roles and permissions for every module. Test: persona-based access tests.</t>
+          <t>System: roles and permissions for every module. Test: persona-based access tests.</t>
         </is>
       </c>
       <c r="H125" s="39" t="inlineStr">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="J126" s="12" t="inlineStr">
         <is>
-          <t>Build once; both rows point to the same reports.</t>
+          <t>One set of reports; both rows point to the same reports.</t>
         </is>
       </c>
       <c r="K126" s="12" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="G127" s="12" t="inlineStr">
         <is>
-          <t>None on the build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H127" s="39" t="inlineStr">
@@ -13903,7 +13903,7 @@
       </c>
       <c r="G128" s="12" t="inlineStr">
         <is>
-          <t>Business: which submitted policies are renewed. Build: bucket rules. Test: classification cases.</t>
+          <t>Business: which submitted policies are renewed. System: bucket rules. Test: classification cases.</t>
         </is>
       </c>
       <c r="H128" s="39" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="G129" s="12" t="inlineStr">
         <is>
-          <t>Build: IAAF structure. Test: IAAF cases.</t>
+          <t>System: IAAF structure. Test: IAAF cases.</t>
         </is>
       </c>
       <c r="H129" s="39" t="inlineStr">
@@ -14057,7 +14057,7 @@
       </c>
       <c r="G130" s="12" t="inlineStr">
         <is>
-          <t>Business: handling-fee income. Build: disposition steps and GL. Test: no criteria.</t>
+          <t>Business: handling-fee income. System: disposition steps and GL. Test: no criteria.</t>
         </is>
       </c>
       <c r="H130" s="39" t="inlineStr">
@@ -14284,7 +14284,7 @@
       </c>
       <c r="G133" s="12" t="inlineStr">
         <is>
-          <t>Business: two renewal paths. Build: one owner for renewal letters and hold cover. Test: duplicated cases.</t>
+          <t>Business: two renewal paths. System: one owner for renewal letters and hold cover. Test: duplicated cases.</t>
         </is>
       </c>
       <c r="H133" s="39" t="inlineStr">
@@ -14361,7 +14361,7 @@
       </c>
       <c r="G134" s="12" t="inlineStr">
         <is>
-          <t>Build: three reports dropped.</t>
+          <t>System: three reports dropped.</t>
         </is>
       </c>
       <c r="H134" s="39" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="J134" s="12" t="inlineStr">
         <is>
-          <t>Rows marked DROPPED; not built.</t>
+          <t>Rows marked DROPPED; not in scope.</t>
         </is>
       </c>
       <c r="K134" s="12" t="inlineStr">
@@ -14438,7 +14438,7 @@
       </c>
       <c r="G135" s="12" t="inlineStr">
         <is>
-          <t>Business: scope expectation. Build: menu structure.</t>
+          <t>Business: scope expectation. System: menu structure.</t>
         </is>
       </c>
       <c r="H135" s="39" t="inlineStr">
@@ -14515,7 +14515,7 @@
       </c>
       <c r="G136" s="12" t="inlineStr">
         <is>
-          <t>Business: scope. Build: no requirements, sources or layouts.</t>
+          <t>Business: scope. System: no requirements, sources or layouts.</t>
         </is>
       </c>
       <c r="H136" s="39" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="G137" s="12" t="inlineStr">
         <is>
-          <t>Build: one platform serves all modules, so the widest window applies and batch windows shrink. Test: availability tests per window.</t>
+          <t>System: one platform serves all modules, so the widest window applies and batch windows shrink. Test: availability tests per window.</t>
         </is>
       </c>
       <c r="H137" s="39" t="inlineStr">
@@ -14665,7 +14665,7 @@
       </c>
       <c r="G138" s="12" t="inlineStr">
         <is>
-          <t>Build: HA design; 99.99% and 100% need a different architecture and cost. Test: availability measurement.</t>
+          <t>System: HA design; 99.99% and 100% need a different architecture and cost. Test: availability measurement.</t>
         </is>
       </c>
       <c r="H138" s="39" t="inlineStr">
@@ -14742,7 +14742,7 @@
       </c>
       <c r="G139" s="12" t="inlineStr">
         <is>
-          <t>Build: backup frequency and DR design follow the strictest RPO. Test: DR drill targets.</t>
+          <t>System: backup frequency and DR design follow the strictest RPO. Test: DR drill targets.</t>
         </is>
       </c>
       <c r="H139" s="39" t="inlineStr">
@@ -14823,7 +14823,7 @@
       </c>
       <c r="G140" s="12" t="inlineStr">
         <is>
-          <t>Business: legal record keeping (AMLA, BIR). Build: retention rules per record type and archive design. Test: purge cases.</t>
+          <t>Business: legal record keeping (AMLA, BIR). System: retention rules per record type and archive design. Test: purge cases.</t>
         </is>
       </c>
       <c r="H140" s="39" t="inlineStr">
@@ -14977,7 +14977,7 @@
       </c>
       <c r="G142" s="12" t="inlineStr">
         <is>
-          <t>Build: no common maintenance slot unless one window is agreed.</t>
+          <t>System: no common maintenance slot unless one window is agreed.</t>
         </is>
       </c>
       <c r="H142" s="39" t="inlineStr">
@@ -15054,7 +15054,7 @@
       </c>
       <c r="G143" s="12" t="inlineStr">
         <is>
-          <t>Build: no values. Test: no targets.</t>
+          <t>System: no values. Test: no targets.</t>
         </is>
       </c>
       <c r="H143" s="39" t="inlineStr">
@@ -15131,7 +15131,7 @@
       </c>
       <c r="G144" s="12" t="inlineStr">
         <is>
-          <t>Build: one session policy. Test: timeout cases.</t>
+          <t>System: one session policy. Test: timeout cases.</t>
         </is>
       </c>
       <c r="H144" s="39" t="inlineStr">
@@ -15208,7 +15208,7 @@
       </c>
       <c r="G145" s="12" t="inlineStr">
         <is>
-          <t>Security: session control for all users. Build: session enforcement.</t>
+          <t>Security: session control for all users. System: session enforcement.</t>
         </is>
       </c>
       <c r="H145" s="39" t="inlineStr">
@@ -15223,7 +15223,7 @@
       </c>
       <c r="J145" s="12" t="inlineStr">
         <is>
-          <t>Session log built; enforcement parked behind a parameter until answered.</t>
+          <t>Session log kept; enforcement is a parameter, off until answered.</t>
         </is>
       </c>
       <c r="K145" s="12" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="G147" s="12" t="inlineStr">
         <is>
-          <t>Security: identity source for all users. Build: directory authentication port. Test: login cases.</t>
+          <t>Security: identity source for all users. System: directory authentication port. Test: login cases.</t>
         </is>
       </c>
       <c r="H147" s="39" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="G148" s="12" t="inlineStr">
         <is>
-          <t>Build: password policy applies only to local accounts if EUA is used.</t>
+          <t>System: password policy applies only to local accounts if EUA is used.</t>
         </is>
       </c>
       <c r="H148" s="39" t="inlineStr">
@@ -15593,7 +15593,7 @@
       </c>
       <c r="G150" s="12" t="inlineStr">
         <is>
-          <t>Business: one loan status or two. Build: one LAMD intake.</t>
+          <t>Business: one loan status or two. System: one LAMD intake.</t>
         </is>
       </c>
       <c r="H150" s="39" t="inlineStr">
@@ -15670,7 +15670,7 @@
       </c>
       <c r="G151" s="12" t="inlineStr">
         <is>
-          <t>Build: one or two roles; data visible to each.</t>
+          <t>System: one or two roles; data visible to each.</t>
         </is>
       </c>
       <c r="H151" s="39" t="inlineStr">
@@ -15747,7 +15747,7 @@
       </c>
       <c r="G152" s="12" t="inlineStr">
         <is>
-          <t>Security: document confidentiality. Build: access classes per document type.</t>
+          <t>Security: document confidentiality. System: access classes per document type.</t>
         </is>
       </c>
       <c r="H152" s="39" t="inlineStr">
@@ -15819,12 +15819,12 @@
       </c>
       <c r="F153" s="12" t="inlineStr">
         <is>
-          <t>Report List #135 "Renewal Persistency" is tagged "Renewal/Submitted Policy". The Renewal BRD has no persistency report; only the submitted-accounts part is designed.</t>
+          <t>Report List #135 "Renewal Persistency" is tagged "Renewal/Submitted Policy". The Renewal BRD has no persistency report; only the submitted-accounts part is specified.</t>
         </is>
       </c>
       <c r="G153" s="12" t="inlineStr">
         <is>
-          <t>Build: no owner or layout for the general report.</t>
+          <t>System: no owner or layout for the general report.</t>
         </is>
       </c>
       <c r="H153" s="39" t="inlineStr">
@@ -15901,7 +15901,7 @@
       </c>
       <c r="G154" s="12" t="inlineStr">
         <is>
-          <t>Build: renewal decision matrix cannot test total loss automatically.</t>
+          <t>System: renewal decision matrix cannot test total loss automatically.</t>
         </is>
       </c>
       <c r="H154" s="39" t="inlineStr">
@@ -15978,7 +15978,7 @@
       </c>
       <c r="G155" s="12" t="inlineStr">
         <is>
-          <t>Build: EB programmes must be excluded from the general renewal lists.</t>
+          <t>System: EB programmes must be excluded from the general renewal lists.</t>
         </is>
       </c>
       <c r="H155" s="39" t="inlineStr">
@@ -16055,7 +16055,7 @@
       </c>
       <c r="G156" s="12" t="inlineStr">
         <is>
-          <t>Build: file drop targets. Test: delivery cases.</t>
+          <t>System: file drop targets. Test: delivery cases.</t>
         </is>
       </c>
       <c r="H156" s="39" t="inlineStr">
@@ -16132,7 +16132,7 @@
       </c>
       <c r="G157" s="12" t="inlineStr">
         <is>
-          <t>Business: clients cannot open documents without a known rule. Build: password policy per document type. Test: protection cases.</t>
+          <t>Business: clients cannot open documents without a known rule. System: password policy per document type. Test: protection cases.</t>
         </is>
       </c>
       <c r="H157" s="39" t="inlineStr">
@@ -16209,7 +16209,7 @@
       </c>
       <c r="G158" s="12" t="inlineStr">
         <is>
-          <t>Build: upload validation. Test: file cases.</t>
+          <t>System: upload validation. Test: file cases.</t>
         </is>
       </c>
       <c r="H158" s="39" t="inlineStr">
@@ -16286,7 +16286,7 @@
       </c>
       <c r="G159" s="12" t="inlineStr">
         <is>
-          <t>Business: uncovered risk after expiry. Build: hold cover monitoring. Test: expiry cases.</t>
+          <t>Business: uncovered risk after expiry. System: hold cover monitoring. Test: expiry cases.</t>
         </is>
       </c>
       <c r="H159" s="39" t="inlineStr">
@@ -16363,7 +16363,7 @@
       </c>
       <c r="G160" s="12" t="inlineStr">
         <is>
-          <t>Build: reference formats; matching keys of insurer and LAMD files.</t>
+          <t>System: reference formats; matching keys of insurer and LAMD files.</t>
         </is>
       </c>
       <c r="H160" s="39" t="inlineStr">
@@ -16440,7 +16440,7 @@
       </c>
       <c r="G161" s="12" t="inlineStr">
         <is>
-          <t>Business: go-live readiness. Build: migration loads. Test: reconciliation.</t>
+          <t>Business: go-live readiness. System: migration loads. Test: reconciliation.</t>
         </is>
       </c>
       <c r="H161" s="39" t="inlineStr">
@@ -16521,7 +16521,7 @@
       </c>
       <c r="G162" s="12" t="inlineStr">
         <is>
-          <t>Build: ageing configuration. Test: report totals per bucket.</t>
+          <t>System: ageing configuration. Test: report totals per bucket.</t>
         </is>
       </c>
       <c r="H162" s="39" t="inlineStr">
@@ -16748,7 +16748,7 @@
       </c>
       <c r="G165" s="12" t="inlineStr">
         <is>
-          <t>Build: Word renderer for reports.</t>
+          <t>System: Word renderer for reports.</t>
         </is>
       </c>
       <c r="H165" s="39" t="inlineStr">
@@ -16825,7 +16825,7 @@
       </c>
       <c r="G166" s="12" t="inlineStr">
         <is>
-          <t>Build: report owner.</t>
+          <t>System: report owner.</t>
         </is>
       </c>
       <c r="H166" s="39" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="G167" s="12" t="inlineStr">
         <is>
-          <t>Build: a CSF case module or not.</t>
+          <t>System: a CSF case module or not.</t>
         </is>
       </c>
       <c r="H167" s="39" t="inlineStr">
@@ -16979,7 +16979,7 @@
       </c>
       <c r="G168" s="12" t="inlineStr">
         <is>
-          <t>Build: cheque custody in Claims and Cashiering; possible GL impact.</t>
+          <t>System: cheque custody in Claims and Cashiering; possible GL impact.</t>
         </is>
       </c>
       <c r="H168" s="39" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="J168" s="12" t="inlineStr">
         <is>
-          <t>Parked; if yes, a cheque custody register in Claims (V1026-V1029).</t>
+          <t>Parked; if yes, a cheque custody register in Claims.</t>
         </is>
       </c>
       <c r="K168" s="12" t="inlineStr">
@@ -17749,7 +17749,7 @@
       </c>
       <c r="G178" s="12" t="inlineStr">
         <is>
-          <t>New change log (V1091).</t>
+          <t>New change log.</t>
         </is>
       </c>
       <c r="H178" s="39" t="inlineStr">
@@ -17826,7 +17826,7 @@
       </c>
       <c r="G179" s="12" t="inlineStr">
         <is>
-          <t>MIS field catalogue (V1092).</t>
+          <t>MIS field catalogue.</t>
         </is>
       </c>
       <c r="H179" s="39" t="inlineStr">
@@ -17903,7 +17903,7 @@
       </c>
       <c r="G180" s="12" t="inlineStr">
         <is>
-          <t>Insurer page (V1095).</t>
+          <t>Insurer page.</t>
         </is>
       </c>
       <c r="H180" s="39" t="inlineStr">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="G181" s="12" t="inlineStr">
         <is>
-          <t>Report layout and subscriptions (V1093).</t>
+          <t>Report layout and subscriptions.</t>
         </is>
       </c>
       <c r="H181" s="39" t="inlineStr">
@@ -18057,7 +18057,7 @@
       </c>
       <c r="G182" s="12" t="inlineStr">
         <is>
-          <t>Role home page (V1094).</t>
+          <t>Role home page.</t>
         </is>
       </c>
       <c r="H182" s="39" t="inlineStr">
@@ -18211,7 +18211,7 @@
       </c>
       <c r="G184" s="12" t="inlineStr">
         <is>
-          <t>No build.</t>
+          <t>No system work.</t>
         </is>
       </c>
       <c r="H184" s="39" t="inlineStr">
@@ -18442,7 +18442,7 @@
       </c>
       <c r="G187" s="12" t="inlineStr">
         <is>
-          <t>None on build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H187" s="39" t="inlineStr">
@@ -18510,12 +18510,12 @@
       </c>
       <c r="F188" s="12" t="inlineStr">
         <is>
-          <t>Daily batch invoice printing, delivery to insurers by SFTP and delivery report, per insurer; no format or endpoints; BIBS e-mails each service invoice.</t>
+          <t>Daily batch invoice printing, delivery to insurers by SFTP and delivery report, per insurer; no format or SFTP addresses; BIBS e-mails each service invoice.</t>
         </is>
       </c>
       <c r="G188" s="12" t="inlineStr">
         <is>
-          <t>Insurer invoice batch (V1096); SFTP adapter parked.</t>
+          <t>Insurer invoice batch; SFTP delivery on hold.</t>
         </is>
       </c>
       <c r="H188" s="39" t="inlineStr">
@@ -18535,7 +18535,7 @@
       </c>
       <c r="K188" s="12" t="inlineStr">
         <is>
-          <t>Batch format, SFTP endpoints; replaces e-mail?</t>
+          <t>Batch format, SFTP addresses; replaces e-mail?</t>
         </is>
       </c>
       <c r="L188" s="12" t="inlineStr">
@@ -18607,7 +18607,7 @@
       </c>
       <c r="J189" s="12" t="inlineStr">
         <is>
-          <t>No build until defined.</t>
+          <t>No system work until defined.</t>
         </is>
       </c>
       <c r="K189" s="12" t="inlineStr">
@@ -18746,7 +18746,7 @@
       </c>
       <c r="G191" s="12" t="inlineStr">
         <is>
-          <t>None on build; icon set needed (CRQ17).</t>
+          <t>None on the system; icon set needed (CRQ17).</t>
         </is>
       </c>
       <c r="H191" s="39" t="inlineStr">
@@ -18896,7 +18896,7 @@
       </c>
       <c r="G193" s="12" t="inlineStr">
         <is>
-          <t>Business: the migration scope is not agreed. Build: the answers BRD-13 gives to other BRDs (CQ13, CQ07, RQ27, CSQ01) may change at the walk-through. Test: no signed baseline for the migration test cases.</t>
+          <t>Business: the migration scope is not agreed. System: the answers BRD-13 gives to other BRDs (CQ13, CQ07, RQ27, CSQ01) may change at the walk-through. Test: no signed baseline for the migration test cases.</t>
         </is>
       </c>
       <c r="H193" s="39" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="J193" s="12" t="inlineStr">
         <is>
-          <t>Use the draft as the working baseline; start the migration build (wave DM0) after the walk-through and sign-off.</t>
+          <t>Use the draft as the working baseline; start the migration functions after the walk-through and sign-off.</t>
         </is>
       </c>
       <c r="K193" s="12" t="inlineStr">
@@ -18969,7 +18969,7 @@
       </c>
       <c r="G194" s="12" t="inlineStr">
         <is>
-          <t>None on build. The business goals cannot be read as BDOI's answers.</t>
+          <t>None on the system. The business goals cannot be read as BDOI's answers.</t>
         </is>
       </c>
       <c r="H194" s="39" t="inlineStr">
@@ -19115,7 +19115,7 @@
       </c>
       <c r="G196" s="12" t="inlineStr">
         <is>
-          <t>Build: the decision register and gate G1 of the Migration Console. Business: every data object's treatment depends on it. Test: no acceptance rule for BRID 1.1a.</t>
+          <t>System: the decision register and gate G1 of the Migration Console. Business: every data object's treatment depends on it. Test: no acceptance rule for BRID 1.1a.</t>
         </is>
       </c>
       <c r="H196" s="39" t="inlineStr">
@@ -19192,7 +19192,7 @@
       </c>
       <c r="G197" s="12" t="inlineStr">
         <is>
-          <t>Build: load sizing and the cutover window are project assumptions (1,000,000 client rows, 500,000 open-item rows, 48-hour window). Test: performance targets of the dress rehearsal.</t>
+          <t>System: load sizing and the cutover window are project assumptions (1,000,000 client rows, 500,000 open-item rows, 48-hour window). Test: performance targets of the dress rehearsal.</t>
         </is>
       </c>
       <c r="H197" s="39" t="inlineStr">
@@ -19269,7 +19269,7 @@
       </c>
       <c r="G198" s="12" t="inlineStr">
         <is>
-          <t>Build: account import of legacy headers (V823) and endorsements of legacy invoices (booking V873, adjustment). Business: where endorsements of legacy policies are processed after cutover. Test: endorsement scenarios on legacy invoices.</t>
+          <t>System: account import of legacy headers and endorsements of legacy invoices (booking, adjustment). Business: where endorsements of legacy policies are processed after cutover. Test: endorsement scenarios on legacy invoices.</t>
         </is>
       </c>
       <c r="H198" s="39" t="inlineStr">
@@ -19346,7 +19346,7 @@
       </c>
       <c r="G199" s="12" t="inlineStr">
         <is>
-          <t>Build: the object register, layouts and loaders. Business: extract owners cannot be named. Test: reconciliation per object needs the list.</t>
+          <t>System: the object register, layouts and loaders. Business: extract owners cannot be named. Test: reconciliation per object needs the list.</t>
         </is>
       </c>
       <c r="H199" s="39" t="inlineStr">
@@ -19423,7 +19423,7 @@
       </c>
       <c r="G200" s="12" t="inlineStr">
         <is>
-          <t>Build: loaders for objects F07, P04, P05, R09 and V1025 (Claims) stay parked. Business: go-live readiness of Claims, EB, Submitted Policies and Disbursement. Test: migration test scope.</t>
+          <t>System: the migration of objects F07, P04, P05 and R09 stays on hold. Business: go-live readiness of Claims, EB, Submitted Policies and Disbursement. Test: migration test scope.</t>
         </is>
       </c>
       <c r="H200" s="39" t="inlineStr">
@@ -19500,7 +19500,7 @@
       </c>
       <c r="G201" s="12" t="inlineStr">
         <is>
-          <t>Business: GL and sub-ledgers may not agree at go-live. Build: legacy control accounts, clearing account, OPENING journals (V1087, seed V1982). Test: clearing account at 0.00 is a go / no-go criterion.</t>
+          <t>Business: GL and sub-ledgers may not agree at go-live. System: legacy control accounts, clearing account, OPENING journals. Test: clearing account at 0.00 is a go / no-go criterion.</t>
         </is>
       </c>
       <c r="H201" s="39" t="inlineStr">
@@ -19577,7 +19577,7 @@
       </c>
       <c r="G202" s="12" t="inlineStr">
         <is>
-          <t>Build: the DPPR reversal batch and the top-management approval step rest on assumed meanings. Test: acceptance of BRID 5.5 and 7.1.</t>
+          <t>System: the DPPR reversal batch and the top-management approval step rest on assumed meanings. Test: acceptance of BRID 5.5 and 7.1.</t>
         </is>
       </c>
       <c r="H202" s="39" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="G203" s="12" t="inlineStr">
         <is>
-          <t>Business: first months of renewals after go-live. Build: legacy cohorts through LegacyPolicySource, run-off tracker. Test: renewal of a legacy policy.</t>
+          <t>Business: first months of renewals after go-live. System: legacy cohorts given to Renewal with the migrated headers, run-off tracker. Test: renewal of a legacy policy.</t>
         </is>
       </c>
       <c r="H203" s="39" t="inlineStr">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="G204" s="12" t="inlineStr">
         <is>
-          <t>Build: cutover plan, go / no-go and runbook in the Migration Console. Business: cutover calendar and freeze. Test: trial migrations and dress rehearsal.</t>
+          <t>System: cutover plan, go / no-go and runbook in the Migration Console. Business: cutover calendar and freeze. Test: trial migrations and dress rehearsal.</t>
         </is>
       </c>
       <c r="H204" s="39" t="inlineStr">
@@ -19808,7 +19808,7 @@
       </c>
       <c r="G205" s="12" t="inlineStr">
         <is>
-          <t>None on build.</t>
+          <t>None on the system.</t>
         </is>
       </c>
       <c r="H205" s="39" t="inlineStr">
@@ -19885,7 +19885,7 @@
       </c>
       <c r="G206" s="12" t="inlineStr">
         <is>
-          <t>Build: a write-back transport for ContactSyncGateway, or none. Test: coexistence cases in CSF.</t>
+          <t>System: a write-back transfer from CSF to legacy, or none. Test: coexistence cases in CSF.</t>
         </is>
       </c>
       <c r="H206" s="39" t="inlineStr">
@@ -19900,7 +19900,7 @@
       </c>
       <c r="J206" s="12" t="inlineStr">
         <is>
-          <t>Legacy read-only from cutover; the CSF outbox stays NOT_CONFIGURED; accounts that exist only in legacy are found through LegacyAccountLookup.</t>
+          <t>Legacy read-only from cutover; the CSF outbox stays NOT_CONFIGURED; accounts that exist only in legacy are found through the legacy account lookup.</t>
         </is>
       </c>
       <c r="K206" s="12" t="inlineStr">
@@ -19962,7 +19962,7 @@
       </c>
       <c r="G207" s="12" t="inlineStr">
         <is>
-          <t>Business: collectors lose open promises at cutover. Build: legacy item state loader (V1007). Test: worklist of legacy invoices.</t>
+          <t>Business: collectors lose open promises at cutover. System: legacy item state migration. Test: worklist of legacy invoices.</t>
         </is>
       </c>
       <c r="H207" s="39" t="inlineStr">
@@ -20039,7 +20039,7 @@
       </c>
       <c r="G208" s="12" t="inlineStr">
         <is>
-          <t>Business: receipt books and BIR reporting. Build: migrated UPP creation. Test: UPP intake.</t>
+          <t>Business: receipt books and BIR reporting. System: migrated UPP creation. Test: UPP intake.</t>
         </is>
       </c>
       <c r="H208" s="39" t="inlineStr">
@@ -20116,7 +20116,7 @@
       </c>
       <c r="G209" s="12" t="inlineStr">
         <is>
-          <t>Business: income recognition of unclaimed collections. Build: new disposition with a two-step approval. Test: reclass and reversal.</t>
+          <t>Business: income recognition of unclaimed collections. System: new disposition with a two-step approval. Test: reclass and reversal.</t>
         </is>
       </c>
       <c r="H209" s="39" t="inlineStr">
@@ -20193,7 +20193,7 @@
       </c>
       <c r="G210" s="12" t="inlineStr">
         <is>
-          <t>Business: GL entries on legacy DP and CWT items. Build: DPPR and PR2307 reversal batches. Test: reversal entries.</t>
+          <t>Business: GL entries on legacy DP and CWT items. System: DPPR and PR2307 reversal batches. Test: reversal entries.</t>
         </is>
       </c>
       <c r="H210" s="39" t="inlineStr">
@@ -20208,7 +20208,7 @@
       </c>
       <c r="J210" s="12" t="inlineStr">
         <is>
-          <t>Batches built from an upload or from the Collections "for reversal" tags of legacy invoices, with maker-checker approval; the commission receivable entry per BDOI answer.</t>
+          <t>Batches from an upload or from the Collections "for reversal" tags of legacy invoices, with maker-checker approval; the commission receivable entry per BDOI answer.</t>
         </is>
       </c>
       <c r="K210" s="12" t="inlineStr">
@@ -20270,7 +20270,7 @@
       </c>
       <c r="G211" s="12" t="inlineStr">
         <is>
-          <t>Build: invoice key rule and "open-balance mode" of the intake. Test: component reconciliation.</t>
+          <t>System: invoice key rule and "open-balance mode" of the intake. Test: component reconciliation.</t>
         </is>
       </c>
       <c r="H211" s="39" t="inlineStr">
@@ -20347,7 +20347,7 @@
       </c>
       <c r="G212" s="12" t="inlineStr">
         <is>
-          <t>Compliance: screening coverage at go-live. Build: screening trigger suppression for migrated clients and a full re-screen. Test: screening of the migrated population.</t>
+          <t>Compliance: screening coverage at go-live. System: screening trigger suppression for migrated clients and a full re-screen. Test: screening of the migrated population.</t>
         </is>
       </c>
       <c r="H212" s="39" t="inlineStr">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="G213" s="12" t="inlineStr">
         <is>
-          <t>Business: audit access to legacy history. Build: archive retention and decommissioning criteria. Test: archive inquiry.</t>
+          <t>Business: audit access to legacy history. System: archive retention and decommissioning criteria. Test: archive inquiry.</t>
         </is>
       </c>
       <c r="H213" s="39" t="inlineStr">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="G214" s="12" t="inlineStr">
         <is>
-          <t>Build: counterparties and remittance types in remittance; accounting rules. Test: Drop 1 remittance cases with reinsurance transactions.</t>
+          <t>System: counterparties and remittance types in remittance; accounting rules. Test: Drop 1 remittance cases with reinsurance transactions.</t>
         </is>
       </c>
       <c r="H214" s="39" t="inlineStr">
@@ -20578,7 +20578,7 @@
       </c>
       <c r="G215" s="12" t="inlineStr">
         <is>
-          <t>Build: the portal module and external users are dropped; EB uploads are done by internal users. FRS BRD-8 and its test plan change. IER sizing loses a tenant.</t>
+          <t>System: the portal module and external users are dropped; EB uploads are done by internal users. FRS BRD-8 and its test plan change. IER sizing loses a tenant.</t>
         </is>
       </c>
       <c r="H215" s="39" t="inlineStr">
@@ -20622,7 +20622,7 @@
         </is>
       </c>
     </row>
-    <row r="216" ht="79.59999999999999" customHeight="1">
+    <row r="216" ht="67" customHeight="1">
       <c r="A216" s="38" t="inlineStr">
         <is>
           <t>DCR-212</t>
@@ -20650,12 +20650,12 @@
       </c>
       <c r="F216" s="12" t="inlineStr">
         <is>
-          <t>Drop 2 lists "Marketing Collection (extraction)". BRD-4 Collections is built as a BIBS module fed by the Operations invoice ledger, replacing the separate Collection Management System that legacy fed nightly. "Extraction" suggests a feed from BIBS to a separate collection application.</t>
+          <t>Drop 2 lists "Marketing Collection (extraction)". BRD-4 Collections is a BIBS module fed by the Operations invoice ledger, replacing the separate Collection Management System that legacy fed nightly. "Extraction" suggests a feed from BIBS to a separate collection application.</t>
         </is>
       </c>
       <c r="G216" s="12" t="inlineStr">
         <is>
-          <t>Build: an outbound extraction only if a separate system remains. Test: which drop tests BRD-4.</t>
+          <t>System: an outbound extraction only if a separate system remains. Test: which drop tests BRD-4.</t>
         </is>
       </c>
       <c r="H216" s="39" t="inlineStr">
@@ -20699,7 +20699,7 @@
         </is>
       </c>
     </row>
-    <row r="217" ht="79.59999999999999" customHeight="1">
+    <row r="217" ht="67" customHeight="1">
       <c r="A217" s="38" t="inlineStr">
         <is>
           <t>DCR-213</t>
@@ -20727,7 +20727,7 @@
       </c>
       <c r="F217" s="12" t="inlineStr">
         <is>
-          <t>BRD-10 Sanction Screening and Risk Profiling (built) and the Customer Servicing Facility service-request functions of BRD-9 (designed) are not placed in any drop; only "Account Creation and Maintenance (NB, CSF)" names CSF, and Bridger Insight XG appears among the Drop 2 integrations.</t>
+          <t>BRD-10 Sanction Screening and Risk Profiling and the Customer Servicing Facility service-request functions of BRD-9 are not placed in any drop; only "Account Creation and Maintenance (NB, CSF)" names CSF, and Bridger Insight XG appears among the Drop 2 integrations.</t>
         </is>
       </c>
       <c r="G217" s="12" t="inlineStr">
@@ -21025,7 +21025,7 @@
       </c>
       <c r="D221" s="12" t="inlineStr">
         <is>
-          <t>Programme timeline slide (go-live marker at the end of January 2028; bars); BDOI_DROP_PLAN.md timeline table; BRD-13 design section 17.2</t>
+          <t>Programme timeline slide (go-live marker at the end of January 2028; bars); BDOI drop plan, timeline table; BRD-13 migration strategy, cutover</t>
         </is>
       </c>
       <c r="E221" s="12" t="inlineStr">
@@ -21040,7 +21040,7 @@
       </c>
       <c r="G221" s="12" t="inlineStr">
         <is>
-          <t>Cut-over calendar, year-end close in legacy, GL opening (January stub period if T is later), trial-migration dates.</t>
+          <t>Cut-over calendar, year-end close in legacy, GL opening (a short January period if T is later), trial-migration dates.</t>
         </is>
       </c>
       <c r="H221" s="39" t="inlineStr">
@@ -21117,7 +21117,7 @@
       </c>
       <c r="G222" s="12" t="inlineStr">
         <is>
-          <t>None on the build if the paper is withdrawn; otherwise a separate production release, early client migration and a five-month legacy-to-BIBS client sync.</t>
+          <t>None on the system if the paper is withdrawn; otherwise a separate production release, early client migration and a five-month legacy-to-BIBS client sync.</t>
         </is>
       </c>
       <c r="H222" s="39" t="inlineStr">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="G223" s="12" t="inlineStr">
         <is>
-          <t>Build: code map set and a renewal sanitation check. Test: sample RMEL validation in Trial migration 1.</t>
+          <t>System: code map set and a renewal sanitation check. Test: sample RMEL validation in Trial migration 1.</t>
         </is>
       </c>
       <c r="H223" s="39" t="inlineStr">
@@ -21264,7 +21264,7 @@
       </c>
       <c r="D224" s="12" t="inlineStr">
         <is>
-          <t>Concept paper IV (p.1); BRD-13 BRID 12.1; renewal lead time 140 days (RENEWAL_DESIGN section 9)</t>
+          <t>Concept paper IV (p.1); BRD-13 BRID 12.1; renewal lead time 140 days (FRS BRD-6)</t>
         </is>
       </c>
       <c r="E224" s="12" t="inlineStr">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="G224" s="12" t="inlineStr">
         <is>
-          <t>Business: no lapse of cover over the cut-over. Build: P03 carry-forward.</t>
+          <t>Business: no lapse of cover over the cut-over. System: P03 carry-forward.</t>
         </is>
       </c>
       <c r="H224" s="39" t="inlineStr">
@@ -21437,7 +21437,7 @@
       </c>
       <c r="G226" s="12" t="inlineStr">
         <is>
-          <t>Infrastructure sizing and cost; security and network design; the IER diagram would be signed off for a system that is not built.</t>
+          <t>Infrastructure sizing and cost; security and network design; the IER diagram would be signed off for an architecture BIBS does not use.</t>
         </is>
       </c>
       <c r="H226" s="39" t="inlineStr">
@@ -21452,12 +21452,12 @@
       </c>
       <c r="J226" s="12" t="inlineStr">
         <is>
-          <t>Proposed: BIBS modular monolith with IER enterprise elements (edge security, managed AWS services, separate web, jobs and integration workloads), docs/architecture/ARCHITECTURE_OPTION_DECISION.md, awaiting BDOI confirmation. Replace the IER diagrams with the BIBS application and deployment diagrams (alignment document figures 3 and 4); restate the K8s sheets for the BIBS workloads.</t>
+          <t>Proposed: BIBS modular monolith with IER enterprise elements (edge security, managed AWS services, separate web, jobs and integration workloads), per the architecture option decision, awaiting BDOI confirmation. Replace the IER diagrams with the BIBS application and deployment diagrams (alignment document figures 3 and 4); restate the K8s sheets for the BIBS workloads.</t>
         </is>
       </c>
       <c r="K226" s="12" t="inlineStr">
         <is>
-          <t>Please confirm that the IER will describe BIBS as built, and name the mandatory edge component (ALB + WAF, CloudFront, Apigee X).</t>
+          <t>Please confirm that the IER will describe the BIBS architecture, and name the mandatory edge component (ALB + WAF, CloudFront, Apigee X).</t>
         </is>
       </c>
       <c r="L226" s="12" t="inlineStr">
@@ -21529,7 +21529,7 @@
       </c>
       <c r="J227" s="12" t="inlineStr">
         <is>
-          <t>Proposed: BIBS modular monolith with IER enterprise elements (edge security, managed AWS services, separate web, jobs and integration workloads), docs/architecture/ARCHITECTURE_OPTION_DECISION.md, awaiting BDOI confirmation. BDOI IT corrects the formula (or removes EFS), adds Pre-Prod and DR cluster sheets, fills the environment sheets from the alignment sizing and re-costs.</t>
+          <t>Proposed: BIBS modular monolith with IER enterprise elements (edge security, managed AWS services, separate web, jobs and integration workloads), per the architecture option decision, awaiting BDOI confirmation. BDOI IT corrects the formula (or removes EFS), adds Pre-Prod and DR cluster sheets, fills the environment sheets from the alignment sizing and re-costs.</t>
         </is>
       </c>
       <c r="K227" s="12" t="inlineStr">
@@ -21576,7 +21576,7 @@
       </c>
       <c r="D228" s="12" t="inlineStr">
         <is>
-          <t>IER workbook v20, VDI Requirements (OpenJDK Temurin 17, Node.js 20, Angular), HW &amp; SW Requirements ("RHEL 9.x + PostgreSQL 16 (Amazon RDS)", GitLab Runner), Architecture Diagram (Infra) (a second CI toolchain named in the IER), Architecture Diagram (ArgoCD, Terraform + Crossplane), K8s sheets (Dynatrace)</t>
+          <t>IER workbook v20, VDI Requirements (OpenJDK Temurin 17, Node 20, Angular), HW &amp; SW Requirements ("RHEL 9.x + PostgreSQL 16 (Amazon RDS)", GitLab Runner), Architecture Diagram (Infra) (a second CI toolchain named in the IER), Architecture Diagram (ArgoCD, Terraform + Crossplane), K8s sheets (Dynatrace)</t>
         </is>
       </c>
       <c r="E228" s="12" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="F228" s="12" t="inlineStr">
         <is>
-          <t>The IER names JDK 17, Node 20 and an Angular SPA; BIBS uses Java 21, Node 22 and React 19. RDS rows name "RHEL 9.x" for a managed engine. Three CI/CD toolchains are named (GitLab, a second CI toolchain named in the IER, ArgoCD) and two observability stacks (Dynatrace; CloudWatch, X-Ray, Prometheus, Loki, Grafana). BIBS builds on the CI pipeline (GitLab CI definition in the delivery) and exposes Prometheus metrics.</t>
+          <t>The IER names JDK 17, Node 20 and an Angular SPA; BIBS uses Java 21, Node 22 and React 19. RDS rows name "RHEL 9.x" for a managed engine. Three CI/CD toolchains are named (GitLab, a second CI toolchain named in the IER, ArgoCD) and two observability stacks (Dynatrace; CloudWatch, X-Ray, Prometheus, Loki, Grafana). BIBS is delivered through one pipeline and exposes Prometheus metrics.</t>
         </is>
       </c>
       <c r="G228" s="12" t="inlineStr">
@@ -21730,7 +21730,7 @@
       </c>
       <c r="D230" s="12" t="inlineStr">
         <is>
-          <t>IER workbook v20, Assumptions 3 (non-production 12 x 5); BIBS job schedules (application.yml)</t>
+          <t>IER workbook v20, Assumptions 3 (non-production 12 x 5); BIBS job schedules (FRS configuration chapters)</t>
         </is>
       </c>
       <c r="E230" s="12" t="inlineStr">
@@ -21807,7 +21807,7 @@
       </c>
       <c r="D231" s="12" t="inlineStr">
         <is>
-          <t>BDOI answer A4 (26-Sep-2026); IER HW &amp; SW Requirements (S3 document store + EFS shared PV); DOCUMENT_STORAGE_DECISION.md</t>
+          <t>BDOI answer A4 (26-Sep-2026); IER HW &amp; SW Requirements (S3 document store + EFS shared PV); document storage proposal</t>
         </is>
       </c>
       <c r="E231" s="12" t="inlineStr">
@@ -21822,7 +21822,7 @@
       </c>
       <c r="G231" s="12" t="inlineStr">
         <is>
-          <t>Build items ST0 (storage port, stored_file, presigned links) and ST1 (every module moved, existing bytes copied); IER rows for buckets, KMS, endpoint, replication and malware scanning; EFS removed.</t>
+          <t>S3 document store and the copy of the existing files; IER rows for buckets, KMS, VPC gateway, replication and malware scanning; EFS removed.</t>
         </is>
       </c>
       <c r="H231" s="39" t="inlineStr">
@@ -21837,12 +21837,12 @@
       </c>
       <c r="J231" s="12" t="inlineStr">
         <is>
-          <t>Option C of DOCUMENT_STORAGE_DECISION.md: S3 for bytes, PostgreSQL metadata, 5-minute presigned links after the permission check and audit, four buckets per environment, SSE-KMS, Object Lock governance, cross-region replication.</t>
+          <t>Option C of the document storage proposal: S3 for the file content, PostgreSQL metadata, 5-minute signed links after the permission check and audit, four buckets per environment, SSE-KMS, Object Lock governance, cross-region replication.</t>
         </is>
       </c>
       <c r="K231" s="12" t="inlineStr">
         <is>
-          <t>Please confirm option C and the five decisions of DOCUMENT_STORAGE_DECISION.md section 5.</t>
+          <t>Please confirm option C and the five decisions of the document storage proposal.</t>
         </is>
       </c>
       <c r="L231" s="12" t="inlineStr">
@@ -21980,7 +21980,7 @@
       </c>
       <c r="G233" s="12" t="inlineStr">
         <is>
-          <t>Build: provisioning API and aggregation; the BRD-11 request screens may be reduced. Test: joiner / mover / leaver cases.</t>
+          <t>System: provisioning API and aggregation; the BRD-11 request screens may be reduced. Test: joiner / mover / leaver cases.</t>
         </is>
       </c>
       <c r="H233" s="39" t="inlineStr">
@@ -22057,7 +22057,7 @@
       </c>
       <c r="G234" s="12" t="inlineStr">
         <is>
-          <t>Build: OIDC sign-in in the frontend and backend, user mapping, break-glass administrator; lockout and password rules move to Entra ID. Test: log-in cases of every BRD.</t>
+          <t>System: OIDC sign-in in the frontend and backend, user mapping, break-glass administrator; lockout and password rules move to Entra ID. Test: log-in cases of every BRD.</t>
         </is>
       </c>
       <c r="H234" s="39" t="inlineStr">
@@ -22134,7 +22134,7 @@
       </c>
       <c r="G235" s="12" t="inlineStr">
         <is>
-          <t>Delivery model of the build and support teams; VDI count.</t>
+          <t>Delivery model of the delivery and support teams; VDI count.</t>
         </is>
       </c>
       <c r="H235" s="39" t="inlineStr">
@@ -22288,7 +22288,7 @@
       </c>
       <c r="G237" s="12" t="inlineStr">
         <is>
-          <t>Build: two new outbound interfaces in Drop 2 (build Mar-Apr 2027). Test: reconciliation of EGL to the BIBS GL.</t>
+          <t>System: two new outbound interfaces in Drop 2 (Mar-Apr 2027). Test: reconciliation of EGL to the BIBS GL.</t>
         </is>
       </c>
       <c r="H237" s="39" t="inlineStr">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="G238" s="12" t="inlineStr">
         <is>
-          <t>Build: layouts and possibly host-to-host transfer in Drop 0.</t>
+          <t>System: layouts and possibly host-to-host transfer in Drop 0.</t>
         </is>
       </c>
       <c r="H238" s="39" t="inlineStr">
@@ -22380,7 +22380,7 @@
       </c>
       <c r="J238" s="12" t="inlineStr">
         <is>
-          <t>Layouts configured in the payment-file layout table; CMS / New BOB outward file built in disbursement; automated transfer if BDOI IT offers it.</t>
+          <t>Layouts configured in the payment-file layout table; CMS / New BOB outward file from Disbursement; automated transfer if BDOI IT offers it.</t>
         </is>
       </c>
       <c r="K238" s="12" t="inlineStr">
@@ -22519,7 +22519,7 @@
       </c>
       <c r="G240" s="12" t="inlineStr">
         <is>
-          <t>Business: renewals of January-May 2028 expiries (about 25,800 accounts a month, umbrella p.44-45). Build: carried RMEL cohorts (layout P03), catch-up extraction in Renewal, no pre-cut-over production load. Test: renewal of a carried legacy policy; trial-migration load order.</t>
+          <t>Business: renewals of January-May 2028 expiries (about 25,800 accounts a month, umbrella p.44-45). System: carried RMEL cohorts (layout P03), catch-up extraction in Renewal, no pre-cut-over production load. Test: renewal of a carried legacy policy; trial-migration load order.</t>
         </is>
       </c>
       <c r="H240" s="39" t="inlineStr">
@@ -22534,7 +22534,7 @@
       </c>
       <c r="J240" s="12" t="inlineStr">
         <is>
-          <t>Concept paper recorded as superseded by the single January 2028 go-live. Kept from it: reference data and clients load first in every trial migration (prerequisite for renewal testing); RMEL validation and exception handling for the carried January-May 2028 cohorts; the package remapping decision. Proposal for the cohorts: prepared in legacy from August 2027 as today, carried at the freeze with their disposition, placed and booked in BIBS from go-live; catch-up extraction at go-live as the safety net (DATA_MIGRATION_DESIGN section 15.1).</t>
+          <t>Concept paper recorded as superseded by the single January 2028 go-live. Kept from it: reference data and clients load first in every trial migration (prerequisite for renewal testing); RMEL validation and exception handling for the carried January-May 2028 cohorts; the package remapping decision. Proposal for the cohorts: prepared in legacy from August 2027 as today, carried at the freeze with their disposition, placed and booked in BIBS from go-live; catch-up extraction at go-live as the safety net (BRD-13 migration strategy).</t>
         </is>
       </c>
       <c r="K240" s="12" t="inlineStr">
@@ -22600,7 +22600,7 @@
       </c>
       <c r="G241" s="12" t="inlineStr">
         <is>
-          <t>Business: correct package on renewals and endorsements of legacy policies. Build: PACKAGE code map with conditional entries; Renewal sanitation check for unresolved packages. Test: package split by sum-insured band; unresolved package in the Exception bucket.</t>
+          <t>Business: correct package on renewals and endorsements of legacy policies. System: PACKAGE code map with conditional entries; Renewal sanitation check for unresolved packages. Test: package split by sum-insured band; unresolved package in the Exception bucket.</t>
         </is>
       </c>
       <c r="H241" s="39" t="inlineStr">
@@ -22666,7 +22666,7 @@
       </c>
       <c r="D242" s="12" t="inlineStr">
         <is>
-          <t>BDOI Programme Timeline (image, go-live marker at the end of the January 2028 column); BRD-13 BRID 12.1 (p.12); DATA_MIGRATION_DESIGN section 17.2</t>
+          <t>BDOI Programme Timeline (image, go-live marker at the end of the January 2028 column); BRD-13 BRID 12.1 (p.12); BRD-13 migration strategy, cutover</t>
         </is>
       </c>
       <c r="E242" s="12" t="inlineStr">
@@ -22681,7 +22681,7 @@
       </c>
       <c r="G242" s="12" t="inlineStr">
         <is>
-          <t>Business: availability of staff and bank channels over the holidays; year-end closing and audit adjustments. Build: none. Test: dress rehearsal timings.</t>
+          <t>Business: availability of staff and bank channels over the holidays; year-end closing and audit adjustments. System: none. Test: dress rehearsal timings.</t>
         </is>
       </c>
       <c r="H242" s="39" t="inlineStr">
@@ -22762,7 +22762,7 @@
       </c>
       <c r="G243" s="12" t="inlineStr">
         <is>
-          <t>Business: business units must consolidate their disposition files monthly. Build: layout P03 combines the legacy RMEL extract with the disposition file; cohort completeness check. Test: rejected rows in every trial migration.</t>
+          <t>Business: business units must consolidate their disposition files monthly. System: layout P03 combines the legacy RMEL extract with the disposition file; cohort completeness check. Test: rejected rows in every trial migration.</t>
         </is>
       </c>
       <c r="H243" s="39" t="inlineStr">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>For "Invoice Batch Printing" (p.43): what is the batch file (one PDF per insurer, a ZIP, a manifest), the SFTP endpoint per insurer, and does it replace the e-mail of each service invoice?</t>
+          <t>For "Invoice Batch Printing" (p.43): what is the batch file (one PDF per insurer, a ZIP, a manifest), the SFTP address per insurer, and does it replace the e-mail of each service invoice?</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -27707,7 +27707,7 @@
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Are the MKTID activities (hold, special remittance, 2307 tagging, DP tagging, send schedule) delivered in the Operations build or by a Marketing / Collection BRD that will feed Operations?</t>
+          <t>Are the MKTID activities (hold, special remittance, 2307 tagging, DP tagging, send schedule) delivered in the Operations module or by a Marketing / Collection BRD that will feed Operations?</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
@@ -30159,7 +30159,7 @@
       </c>
       <c r="D178" s="12" t="inlineStr">
         <is>
-          <t>For each mode: manual at the branch, BDO BOB, or file (DCTF to TPD for ACA). Full DCTF specification (header / trailer / totals), credited-accounts .txt layout, deposited-checks file layout, BOB approval report; will any channel become an API?</t>
+          <t>For each mode: manual at the branch, BDO BOB, or file (DCTF to TPD for ACA). Full DCTF specification (header / trailer / totals), credited-accounts.txt layout, deposited-checks file layout, BOB approval report; will any channel become an API?</t>
         </is>
       </c>
       <c r="E178" s="12" t="inlineStr">
@@ -39251,7 +39251,7 @@
       </c>
       <c r="D406" s="12" t="inlineStr">
         <is>
-          <t>(Priority 1) Which date in January 2028 is T? We propose Monday 3 January 2028, with the legacy freeze after the EOD of Wednesday 29 December 2027 and the legacy December / year-end close completed in legacy before the final extracts. If T is later in January, the migration rule "first business day of a month after a legacy month-end close" (DMQ25) no longer holds and the GL opening needs a January stub period.</t>
+          <t>(Priority 1) Which date in January 2028 is T? We propose Monday 3 January 2028, with the legacy freeze after the EOD of Wednesday 29 December 2027 and the legacy December / year-end close completed in legacy before the final extracts. If T is later in January, the migration rule "first business day of a month after a legacy month-end close" (DMQ25) no longer holds and the GL opening needs a short January period.</t>
         </is>
       </c>
       <c r="E406" s="12" t="inlineStr">
@@ -40187,7 +40187,7 @@
       </c>
       <c r="D430" s="12" t="inlineStr">
         <is>
-          <t>(Priority 1) Please confirm that the IER describes BIBS as built: one backend (modular monolith) and one frontend on EKS, RDS PostgreSQL 16, ElastiCache Redis 7, MSK Kafka, S3; not the ten bv-* microservices, Aurora / MongoDB, Istio / OPA or EventBridge. Which edge is the BDO standard: ALB + WAF, CloudFront, Apigee X?</t>
+          <t>(Priority 1) Please confirm that the IER describes the BIBS architecture: one backend (modular monolith) and one frontend on EKS, RDS PostgreSQL 16, ElastiCache Redis 7, MSK Kafka, S3; not the ten bv-* microservices, Aurora / MongoDB, Istio / OPA or EventBridge. Which edge is the BDO standard: ALB + WAF, CloudFront, Apigee X?</t>
         </is>
       </c>
       <c r="E430" s="12" t="inlineStr">
@@ -40427,12 +40427,12 @@
       </c>
       <c r="D436" s="12" t="inlineStr">
         <is>
-          <t>(Priority 1) Please confirm the five decisions of DOCUMENT_STORAGE_DECISION.md section 5: option C with 5-minute presigned links (or option B, streaming through BIBS); the malware scanning service; Object Lock mode and the records under legal hold; KMS key ownership and rotation; whether ECM receives copies of any record class. Also the bucket account and the DR region for replication.</t>
+          <t>(Priority 1) Please confirm the five decisions of the document storage proposal: option C with 5-minute presigned links (or option B, streaming through BIBS); the malware scanning service; Object Lock mode and the records under legal hold; KMS key ownership and rotation; whether ECM receives copies of any record class. Also the bucket account and the DR region for replication.</t>
         </is>
       </c>
       <c r="E436" s="12" t="inlineStr">
         <is>
-          <t>Answer A4; DOCUMENT_STORAGE_DECISION.md</t>
+          <t>Answer A4; Document storage proposal</t>
         </is>
       </c>
       <c r="F436" s="32" t="inlineStr">
@@ -40628,7 +40628,7 @@
       </c>
       <c r="E441" s="12" t="inlineStr">
         <is>
-          <t>DOCUMENT_STORAGE_DECISION.md Open points for BDOI IT</t>
+          <t>Document storage proposal Open points for BDOI IT</t>
         </is>
       </c>
       <c r="F441" s="32" t="inlineStr">
@@ -40668,7 +40668,7 @@
       </c>
       <c r="E442" s="12" t="inlineStr">
         <is>
-          <t>DOCUMENT_STORAGE_DECISION.md Open points for BDOI IT</t>
+          <t>Document storage proposal Open points for BDOI IT</t>
         </is>
       </c>
       <c r="F442" s="32" t="inlineStr">
@@ -40708,7 +40708,7 @@
       </c>
       <c r="E443" s="12" t="inlineStr">
         <is>
-          <t>DOCUMENT_STORAGE_DECISION.md Open points for BDOI IT</t>
+          <t>Document storage proposal Open points for BDOI IT</t>
         </is>
       </c>
       <c r="F443" s="32" t="inlineStr">
@@ -40748,7 +40748,7 @@
       </c>
       <c r="E444" s="12" t="inlineStr">
         <is>
-          <t>DOCUMENT_STORAGE_DECISION.md Open points for BDOI IT</t>
+          <t>Document storage proposal Open points for BDOI IT</t>
         </is>
       </c>
       <c r="F444" s="32" t="inlineStr">
@@ -40765,7 +40765,7 @@
         </is>
       </c>
     </row>
-    <row r="445" ht="67" customHeight="1">
+    <row r="445" ht="54.4" customHeight="1">
       <c r="A445" s="12" t="inlineStr">
         <is>
           <t>XQ01</t>
@@ -40783,12 +40783,12 @@
       </c>
       <c r="D445" s="12" t="inlineStr">
         <is>
-          <t>Is it one LAMD report (one file, one owner) or two different reports? Who uploads it? (RQ20, SP SQ06) Background: Renewal uploads LAMD paid-off / RMU reports (RNW_LAMD_REPORT, rnw_lamd_report / rnw_lamd_line, role LAMD); Submitted Policies uploads a LAMD loan snapshot (SBM_LAMD, sbm_lamd_loan). Both match on the PN</t>
+          <t>Is it one LAMD report (one file, one owner) or two different reports? Who uploads it? (RQ20, SP SQ06) Background: Renewal uploads LAMD paid-off / RMU reports (role LAMD); Submitted Policies uploads a LAMD loan snapshot. Both match on the PN</t>
         </is>
       </c>
       <c r="E445" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F445" s="32" t="inlineStr">
@@ -40832,7 +40832,7 @@
       </c>
       <c r="E446" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F446" s="32" t="inlineStr">
@@ -40853,7 +40853,7 @@
         </is>
       </c>
     </row>
-    <row r="447" ht="54.4" customHeight="1">
+    <row r="447" ht="67" customHeight="1">
       <c r="A447" s="12" t="inlineStr">
         <is>
           <t>XQ03</t>
@@ -40871,12 +40871,12 @@
       </c>
       <c r="D447" s="12" t="inlineStr">
         <is>
-          <t>Are the renewal notice and renewal proposal letters part of the renewal (Renewal module) or of the masterlist follow-up (Submitted Policies)? (SP SQ09) Background: sbm_letter types RENEWAL_NOTICE and RENEWAL_PROPOSAL are renewal-related, but D2 names only RA / NRNS / NAL / SFU</t>
+          <t>Are the renewal notice and renewal proposal letters part of the renewal (Renewal module) or of the masterlist follow-up (Submitted Policies)? (SP SQ09) Background: the Submitted Policies letter types RENEWAL_NOTICE and RENEWAL_PROPOSAL are renewal-related, but D2 names only RA / NRNS / NAL / SFU</t>
         </is>
       </c>
       <c r="E447" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F447" s="32" t="inlineStr">
@@ -40920,7 +40920,7 @@
       </c>
       <c r="E448" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F448" s="32" t="inlineStr">
@@ -40959,12 +40959,12 @@
       </c>
       <c r="D449" s="12" t="inlineStr">
         <is>
-          <t>Which claim documents does the contact centre retrieve, and should claim documents use the platform DOCUMENT_TYPE list or BCL_DOCUMENT_TYPE? (CLQ26, CSQ07) Background: Claims keeps its own document-type LOV (BCL_DOCUMENT_TYPE: PLA, CRF, estimate, offer, LOA, release papers ...); CSF expects CLAIM_REPORT</t>
+          <t>Which claim documents does the contact centre retrieve, and should claim documents use the platform DOCUMENT_TYPE list or BCL_DOCUMENT_TYPE? (CLQ26, CSQ07) Background: Claims keeps its own document-type LOV (BCL_DOCUMENT_TYPE: PLA, CRF, estimate, offer, LOA, release papers...); CSF expects CLAIM_REPORT</t>
         </is>
       </c>
       <c r="E449" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F449" s="32" t="inlineStr">
@@ -41003,12 +41003,12 @@
       </c>
       <c r="D450" s="12" t="inlineStr">
         <is>
-          <t>Layout and definition of the general Renewal Persistency Report Background: Report List #135: SP builds SBM-PERSISTENCY for submitted accounts and says the general report belongs to Renewal; the Renewal design has no persistency report</t>
+          <t>Layout and definition of the general Renewal Persistency Report Background: Report List #135: SP proposes SBM-PERSISTENCY for submitted accounts and says the general report belongs to Renewal; the Renewal FRS has no persistency report</t>
         </is>
       </c>
       <c r="E450" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F450" s="32" t="inlineStr">
@@ -41048,7 +41048,7 @@
       </c>
       <c r="E451" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F451" s="32" t="inlineStr">
@@ -41084,7 +41084,7 @@
       </c>
       <c r="E452" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F452" s="32" t="inlineStr">
@@ -41132,7 +41132,7 @@
       </c>
       <c r="E453" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F453" s="32" t="inlineStr">
@@ -41176,7 +41176,7 @@
       </c>
       <c r="E454" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F454" s="32" t="inlineStr">
@@ -41220,7 +41220,7 @@
       </c>
       <c r="E455" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F455" s="32" t="inlineStr">
@@ -41264,7 +41264,7 @@
       </c>
       <c r="E456" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F456" s="32" t="inlineStr">
@@ -41304,7 +41304,7 @@
       </c>
       <c r="E457" s="12" t="inlineStr">
         <is>
-          <t>BDOI_CROSS_BRD_DECISIONS.md section 5</t>
+          <t>Cross-BRD decisions section 5</t>
         </is>
       </c>
       <c r="F457" s="32" t="inlineStr">

</xml_diff>

<commit_message>
Use 'on hold' instead of 'parked' in client documents and rebuild the change register, discrepancy register and process deck
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Registers/BIBS_Register_BRD-00_Discrepancies_and_Clarifications_v1.2.xlsx
+++ b/docs/deliverables/out/Programme/Registers/BIBS_Register_BRD-00_Discrepancies_and_Clarifications_v1.2.xlsx
@@ -12775,7 +12775,7 @@
       </c>
       <c r="J113" s="12" t="inlineStr">
         <is>
-          <t>Screen individuals and corporates against the same lists; NLDS kept as a parked source.</t>
+          <t>Screen individuals and corporates against the same lists; NLDS kept as a source on hold.</t>
         </is>
       </c>
       <c r="K113" s="12" t="inlineStr">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="J124" s="12" t="inlineStr">
         <is>
-          <t>User administration guide in the Help Center; external ACL parked.</t>
+          <t>User administration guide in the Help Center; external ACL on hold.</t>
         </is>
       </c>
       <c r="K124" s="12" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="J168" s="12" t="inlineStr">
         <is>
-          <t>Parked; if yes, a cheque custody register in Claims.</t>
+          <t>On hold; if yes, a cheque custody register in Claims.</t>
         </is>
       </c>
       <c r="K168" s="12" t="inlineStr">
@@ -43071,7 +43071,7 @@
       </c>
       <c r="Q21" s="12" t="inlineStr">
         <is>
-          <t>Several roles per user; single session per device parked until answered</t>
+          <t>Several roles per user; single session per device on hold until answered</t>
         </is>
       </c>
       <c r="R21" s="12" t="inlineStr">

</xml_diff>